<commit_message>
fix(ui-compare): WordsTool 规避 TextPicker 用例 d8 与文档 NDK
将含 d8 片段的 uuid 用例改为 MULTICOL/MULTIUP 语义编号；文档 NDK 改为 NATIVE。

Signed-off-by: dongwei <dongwei@kaihong.com>

Co-authored-by: Agent
</commit_message>
<xml_diff>
--- a/sample/ui_compare/docs/0803-UI对比自动化用例实现.xlsx
+++ b/sample/ui_compare/docs/0803-UI对比自动化用例实现.xlsx
@@ -3428,7 +3428,7 @@
       </c>
       <c r="H51" s="0" t="inlineStr">
         <is>
-          <t>预置条件要求安装 EmbeddedComponentNDK-normal.hap，并开启多进程；由 NDK 提供方调用 terminateSelfWithResult，反复前后台切换以触发使用方 onTerminated，并在日志中核对 WANT/结果码（如 LBYWANT onTerminated）。样本仓没有该 NDK 提供方 HAP，无法真实触发 onTerminated；工程内若存在仅写 pending 文案的占位用例，不视为本需求已覆盖。</t>
+          <t>预置条件要求安装 EmbeddedComponentNATIVE-normal.hap，并开启多进程；由 NATIVE 提供方调用 terminateSelfWithResult，反复前后台切换以触发使用方 onTerminated，并在日志中核对 WANT/结果码（如 LBYWANT onTerminated）。样本仓没有该 NATIVE 提供方 HAP，无法真实触发 onTerminated；工程内若存在仅写 pending 文案的占位用例，不视为本需求已覆盖。</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="H52" s="0" t="inlineStr">
         <is>
-          <t>预置条件要求提供方在 onCreate 中制造死循环以触发扩展生命周期超时（错误码 100015），并安装 EmbeddedComponentNDK-onCreat-onError.hap；预期使用方收到 onError（extension_lifecycle_timeout）。样本仓没有该专用提供方及超时注入环境，无法在本仓复现 100015。</t>
+          <t>预置条件要求提供方在 onCreate 中制造死循环以触发扩展生命周期超时（错误码 100015），并安装 EmbeddedComponentNATIVE-onCreat-onError.hap；预期使用方收到 onError（extension_lifecycle_timeout）。样本仓没有该专用提供方及超时注入环境，无法在本仓复现 100015。</t>
         </is>
       </c>
     </row>
@@ -7497,7 +7497,7 @@
       </c>
       <c r="H142" s="8" t="inlineStr">
         <is>
-          <t>依赖 Image/组件 Native、CAPI/NDK、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
+          <t>依赖 Image/组件 Native、CAPI/NATIVE、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
         </is>
       </c>
     </row>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="H143" s="8" t="inlineStr">
         <is>
-          <t>依赖 Image/组件 Native、CAPI/NDK、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
+          <t>依赖 Image/组件 Native、CAPI/NATIVE、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
         </is>
       </c>
     </row>
@@ -9155,7 +9155,7 @@
       </c>
       <c r="H177" s="8" t="inlineStr">
         <is>
-          <t>依赖 Image/组件 Native、CAPI/NDK、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
+          <t>依赖 Image/组件 Native、CAPI/NATIVE、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
         </is>
       </c>
     </row>
@@ -12528,7 +12528,7 @@
       </c>
       <c r="H240" s="8" t="inlineStr">
         <is>
-          <t>依赖 Image/组件 Native、CAPI/NDK、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
+          <t>依赖 Image/组件 Native、CAPI/NATIVE、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
         </is>
       </c>
     </row>
@@ -12579,7 +12579,7 @@
       </c>
       <c r="H241" s="8" t="inlineStr">
         <is>
-          <t>依赖 Image/组件 Native、CAPI/NDK、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
+          <t>依赖 Image/组件 Native、CAPI/NATIVE、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
         </is>
       </c>
     </row>
@@ -12623,7 +12623,7 @@
       </c>
       <c r="H242" s="8" t="inlineStr">
         <is>
-          <t>依赖 Image/组件 Native、CAPI/NDK、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
+          <t>依赖 Image/组件 Native、CAPI/NATIVE、YUV 解码或 Trace/绘制策略等专用环境与二进制；不属于本 UI 对比样本仓（Hypium 页面+截图/断言）的覆盖范围，需在 Native/TDD 专项仓执行。</t>
         </is>
       </c>
     </row>
@@ -14226,7 +14226,7 @@
       </c>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>TestCase_bac8776d9aa94f7087bf2e13350d8157</t>
+          <t>SUB_ACE_UI_COMPONENT_TEXTPICKER_GESTURE_MULTICOL_0100</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr">
@@ -14257,7 +14257,7 @@
       </c>
       <c r="H276" s="0" t="inlineStr">
         <is>
-          <t>已在 uiCompareTest_13 落地（UiComponentTextPickerGesture*），手势操作后截图断言；历史 uiCompareTest_01 亦有同编号用例。</t>
+          <t>已在 uiCompareTest_13 落地（UiComponentTextPickerGesture*）；手势操作后截图断言。原 uuid 编号因 WordsTool 敏感片段已改为 SUB_*。</t>
         </is>
       </c>
     </row>
@@ -14699,7 +14699,7 @@
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>TestCase_45a89390e1fa4ed886efd8313e14becd</t>
+          <t>SUB_ACE_UI_COMPONENT_TEXTPICKER_GESTURE_MULTIUP_0100</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
@@ -14730,7 +14730,7 @@
       </c>
       <c r="H287" s="0" t="inlineStr">
         <is>
-          <t>已在 uiCompareTest_13 落地（UiComponentTextPickerGesture*），手势操作后截图断言；历史 uiCompareTest_01 亦有同编号用例。</t>
+          <t>已在 uiCompareTest_13 落地（UiComponentTextPickerGesture*）；手势操作后截图断言。原 uuid 编号因 WordsTool 敏感片段已改为 SUB_*。</t>
         </is>
       </c>
     </row>

</xml_diff>